<commit_message>
Mark which target companies already have content staff.
Replace the empty product-marketing column with a yes-or-no content check, a contact, and a high, medium, or low chance they need an outside writer.

Co-authored-by: nicolasmpicard-gif <nicolasmpicard-gif@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Supply-chain-climate-company-targets.xlsx
+++ b/Supply-chain-climate-company-targets.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Companies" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Companies'!$A$1:$K$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Companies'!$A$1:$M$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,8 +48,19 @@
       <name val="Calibri"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A1A1A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -66,8 +77,28 @@
         <fgColor rgb="00F3F6F4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EDE3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEEEEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBF3D5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -89,11 +120,25 @@
         <color rgb="00D5DDD8"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9E2DC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9E2DC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E2DC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2DC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -106,6 +151,27 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -486,16 +552,18 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="220" customHeight="1">
+    <row r="2" ht="280" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>This is a working target list, not a census of every company in the world. It covers firms that sell supplier compliance, traceability, or carbon-data software and that publish in English or French. Plan A, Cozero, Climatiq, Vaayu, and carbmee are included.
 Names were checked against company pages, news reports, and public profiles in October 2026. People change jobs. Before you email, confirm the person still works there.
-Heads of product marketing are almost never named on the public site. The column says 'Not publicly listed' on purpose. Search LinkedIn for Head of Product Marketing, Head of Content, or Content Marketing Manager at that company. If none exists, write to the founder.
+Own content? is Yes when a public profile showed someone who writes or manages content: a content manager, a communications lead, or a marketing lead who says they own the content. It is also Yes for a large company where a content team should be assumed until LinkedIn shows an empty seat. No means that check did not find such a person.
+Contact point is who to write, or the reason not to write. Probability is how likely they are to need an outside writer for a white paper or a case study. High means a thin or empty content seat and a company that can still pay. Medium means a generalist already covers content, the company is very small, or an acquisition may have frozen the budget. Low means a content person or a content team already covers this work, or the company is a former employer.
+Start with the High rows. On a Low row, write only when you can name one missing page, such as a French version or a case study they have not published.
 Where a founder could not be confirmed from a page opened for this list, the cell says so. Do not guess. Open the about page and fill the name yourself.
 Use the Content page column to find one specific article, then mention that article in the email and propose one title.
 IntegrityNext and OpenSC are former employers. Do not attach or describe confidential client work.
-Filter the Category column. Start with Carbon data and Supplier compliance in France, the UK, and Berlin. Traceability is the same buyer only when the product is about proof of origin or supplier data.</t>
+Filter the Probability column. Start with High, in carbon data and supplier compliance, in France, the UK, and Berlin. Traceability is the same buyer only when the product is about proof of origin or supplier data.</t>
         </is>
       </c>
     </row>
@@ -510,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -519,11 +587,13 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="58" customWidth="1" min="9" max="9"/>
-    <col width="78" customWidth="1" min="10" max="10"/>
-    <col width="62" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="58" customWidth="1" min="11" max="11"/>
+    <col width="78" customWidth="1" min="12" max="12"/>
+    <col width="62" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -557,33 +627,43 @@
           <t>Founders</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>Head of product marketing</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Own content?</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Contact point</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Probability</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Company page</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Content page</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>What they do</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Check before you email</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -614,33 +694,43 @@
           <t>Lubomila Jordanova</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Lubomila Jordanova, founder. Head of Content Mina Awad left in August 2025. Confirm the seat is still empty. Diginex has acquired the company.</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>https://plana.earth</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>https://plana.earth/academy</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="L2" s="7" t="inlineStr">
         <is>
           <t>Carbon accounting and decarbonisation software for companies.</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="M2" s="7" t="inlineStr">
         <is>
           <t>Confirm whether a co-founder besides Lubomila Jordanova is the right first contact.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1">
+    <row r="3" ht="72" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -671,29 +761,39 @@
           <t>Helen Tacke, Fabian Schwarzer, Tiago Taveira</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>Mariel Garcia, Marketing and Communications Lead. Etienne Manière is Head of Go-to-Market. Marketing is about two people.</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>https://www.cozero.io</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>https://www.cozero.io/blog</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>Carbon management software for measuring, reducing, and reporting corporate and product emissions.</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr"/>
-    </row>
-    <row r="4" ht="48" customHeight="1">
+      <c r="M3" s="10" t="inlineStr"/>
+    </row>
+    <row r="4" ht="72" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -724,29 +824,39 @@
           <t>Hessam Lavi, Philipp von Bieberstein, Isis T. Baulig</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Madeleine Ralph, Content Marketing Manager. Jamie Bolland is Director of Marketing.</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>https://www.climatiq.io</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>https://www.climatiq.io/blog</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="L4" s="7" t="inlineStr">
         <is>
           <t>Emission-factor data and carbon calculation tools that other software can plug into.</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5" ht="48" customHeight="1">
+      <c r="M4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -777,29 +887,39 @@
           <t>Namrata Sandhu, Luca Schmid</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>Hannah Hamilton, Head of Communications. Jen Latimer is listed as Senior Copywriter on the editorial page.</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
         <is>
           <t>https://www.vaayu.tech</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="K5" s="10" t="inlineStr">
         <is>
           <t>https://www.vaayu.tech/insights/</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="L5" s="10" t="inlineStr">
         <is>
           <t>Automated environmental-impact software built for retailers.</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6" ht="48" customHeight="1">
+      <c r="M5" s="10" t="inlineStr"/>
+    </row>
+    <row r="6" ht="72" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -830,33 +950,43 @@
           <t>Christian Heinrich, Robin Spickers</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Lea Manthey, VP Marketing. No current content manager found. The previous content manager left in 2023.</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
         <is>
           <t>https://www.carbmee.com</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>https://www.carbmee.com/knowledge-insights</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="L6" s="7" t="inlineStr">
         <is>
           <t>Product and supply-chain carbon software for emissions-intensive manufacturers.</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="M6" s="7" t="inlineStr">
         <is>
           <t>Also lists a Munich office. Confirm which person still leads the company.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1">
+    <row r="7" ht="72" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -887,33 +1017,43 @@
           <t>Rachel Delacour, Yannick Chaze, Raphael Güller</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Ewa Józefkowicz, Senior Content Marketing Manager.</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
         <is>
           <t>https://www.sweep.net</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="K7" s="10" t="inlineStr">
         <is>
           <t>https://www.sweep.net/blog</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="L7" s="10" t="inlineStr">
         <is>
           <t>Sustainability data software for carbon accounting, supply-chain carbon, and climate disclosure.</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="M7" s="10" t="inlineStr">
         <is>
           <t>Also describes itself as headquartered in Paris and London.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1">
+    <row r="8" ht="72" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -944,33 +1084,43 @@
           <t>Alexis Normand, Arnaud Delubac, Matthieu Vegreville</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Laurent Levrey, VP of Marketing. The team has been hiring its own content person. Write only for a French gap you can name.</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
         <is>
           <t>https://greenly.earth</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>https://greenly.earth/blog</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="L8" s="7" t="inlineStr">
         <is>
           <t>Carbon accounting software for measuring and reducing a company's emissions.</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="M8" s="7" t="inlineStr">
         <is>
           <t>Wikipedia lists Paris. LinkedIn lists New York. Confirm the office you are writing to.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
+    <row r="9" ht="72" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -1001,33 +1151,43 @@
           <t>Laurent Barbezieux, Alex Huyn, Thibault Faninger</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>Mélina Lhermite, Head of Marketing and Communication. She already owns content. Aktio is part of Apave.</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
         <is>
           <t>https://www.aktio.cc</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="K9" s="10" t="inlineStr">
         <is>
           <t>https://www.aktio.cc/ressources</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="L9" s="10" t="inlineStr">
         <is>
           <t>French carbon-accounting software that helps companies measure emissions and plan reductions.</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="M9" s="10" t="inlineStr">
         <is>
           <t>Acquired by Apave in March 2025. Write to the Aktio team, and expect Apave in the process.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1">
+    <row r="10" ht="72" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -1058,33 +1218,43 @@
           <t>Not confirmed in the sources checked for this list</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Manon Le Bourdiec, CMO. SGS took a majority stake in November 2025. Confirm that marketing spend is still open.</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>https://www.sami.eco/en</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>https://www.sami.eco/en/blog</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="L10" s="7" t="inlineStr">
         <is>
           <t>French carbon and ESG software, from a carbon footprint through reporting.</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="M10" s="7" t="inlineStr">
         <is>
           <t>SGS took a majority stake in November 2025. Find the founder on the company site before you email.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1">
+    <row r="11" ht="72" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -1115,33 +1285,43 @@
           <t>Not confirmed in the sources checked for this list</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>Emmanuelle Champy, marketing manager. She already produces guides and customer education.</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
         <is>
           <t>https://www.hellocarbo.com</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="K11" s="10" t="inlineStr">
         <is>
           <t>https://www.hellocarbo.com</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="L11" s="10" t="inlineStr">
         <is>
           <t>French software for carbon footprints, life-cycle assessment, and supplier engagement.</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="M11" s="10" t="inlineStr">
         <is>
           <t>Content is the company site itself. Find a blog or resource URL in the menu before you cite a specific article.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="48" customHeight="1">
+    <row r="12" ht="72" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -1172,33 +1352,43 @@
           <t>Taylor Francis, Avi Itskovich, Christian Anderson</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Meghan Keaney Anderson, who leads product marketing, content, and communications.</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
         <is>
           <t>https://watershed.com</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>https://watershed.com/blog</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="L12" s="7" t="inlineStr">
         <is>
           <t>Enterprise software for corporate carbon accounting and climate programs.</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="M12" s="7" t="inlineStr">
         <is>
           <t>Large team. A content or product-marketing manager is a better first note than a founder.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
+    <row r="13" ht="72" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -1229,33 +1419,43 @@
           <t>Kentaro Kawamori, Jason Offerman, Kim Stroh</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Eliana Cameira has been described on the company blog as Head of Growth Marketing. Confirm she is still in the seat.</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
         <is>
           <t>https://www.persefoni.com</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="K13" s="10" t="inlineStr">
         <is>
           <t>https://www.persefoni.com/insights/blog</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="L13" s="10" t="inlineStr">
         <is>
           <t>Climate management and carbon accounting software for companies and financial institutions.</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="M13" s="10" t="inlineStr">
         <is>
           <t>PitchBook lists Mesa, Arizona. Some profiles say Tempe. Confirm the city on the site.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1">
+    <row r="14" ht="72" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -1286,33 +1486,43 @@
           <t>Kristian Rönn, Adam Wamai Egesa, Robin Undall-Behrend</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Michael Creane, Marketing Content Manager. Greenly and Normative combined in 2026.</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
         <is>
           <t>https://normative.io</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>https://normative.io</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="L14" s="7" t="inlineStr">
         <is>
           <t>Carbon accounting software for corporate greenhouse-gas inventories, including supplier data.</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="M14" s="7" t="inlineStr">
         <is>
           <t>A 2025 company profile said a new CEO had joined. Confirm who leads the company. No separate blog URL was confirmed.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1">
+    <row r="15" ht="72" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Carbon data</t>
@@ -1343,33 +1553,43 @@
           <t>Not confirmed in the sources checked for this list</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Founder — confirm the name on the site. A content-manager job ad has circulated. Confirm whether that seat is still open.</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
         <is>
           <t>https://www.carbonchain.com</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>https://www.carbonchain.com</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="L15" s="10" t="inlineStr">
         <is>
           <t>Supply-chain emissions software, including product footprints and CBAM reporting.</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="M15" s="10" t="inlineStr">
         <is>
           <t>Find the founder and a resource URL on the site before you email.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1">
+    <row r="16" ht="72" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Supplier compliance</t>
@@ -1400,33 +1620,43 @@
           <t>Pierre-François Thaler (co-founder and co-CEO)</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>A content lead. Find the name on LinkedIn. Do not write the co-CEO.</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
         <is>
           <t>https://ecovadis.com</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="K16" s="7" t="inlineStr">
         <is>
           <t>https://resources.ecovadis.com</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="L16" s="7" t="inlineStr">
         <is>
           <t>Ratings and tools for supplier sustainability, risk, and carbon performance.</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="M16" s="7" t="inlineStr">
         <is>
           <t>Large company. Write to a content lead, not the co-CEO, unless you already have an introduction.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
+    <row r="17" ht="72" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Supplier compliance</t>
@@ -1457,33 +1687,43 @@
           <t>Martin Berr-Sorokin, Simon Jaehnig, Nick Heine</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Head of Sustainability Content. Do not pitch. Former employer, and the role already covers white papers, case studies, and regulatory notes in German, English, and French.</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="inlineStr">
         <is>
           <t>https://www.integritynext.com</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="K17" s="10" t="inlineStr">
         <is>
           <t>https://www.integritynext.com/resources/blog</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="L17" s="10" t="inlineStr">
         <is>
           <t>Platform for buyers to monitor supplier sustainability and compliance.</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="M17" s="10" t="inlineStr">
         <is>
           <t>You used to work here. The company site has described Martin Berr-Sorokin as former CEO. Confirm current leadership, and do not use confidential material.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="48" customHeight="1">
+    <row r="18" ht="72" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Supplier compliance</t>
@@ -1514,33 +1754,43 @@
           <t>Not confirmed in the sources checked for this list</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Olivia Thomson, Communications Manager. Maurizio Capuzzo is CMO.</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
         <is>
           <t>https://www.sedex.com</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="K18" s="7" t="inlineStr">
         <is>
           <t>https://www.sedex.com/blog</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="L18" s="7" t="inlineStr">
         <is>
           <t>Membership platform where companies share ethical and responsible-sourcing audit data on suppliers.</t>
         </is>
       </c>
-      <c r="K18" s="4" t="inlineStr">
+      <c r="M18" s="7" t="inlineStr">
         <is>
           <t>Member organisation rather than a classic startup. Find the current content lead.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="48" customHeight="1">
+    <row r="19" ht="72" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Supplier compliance</t>
@@ -1571,29 +1821,39 @@
           <t>Jonathan Hughes (co-founder; other co-founders not confirmed here)</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>A content lead. Find the name on LinkedIn.</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J19" s="10" t="inlineStr">
         <is>
           <t>https://www.assent.com</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="K19" s="10" t="inlineStr">
         <is>
           <t>https://www.assent.com/resources/content-hub/</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="L19" s="10" t="inlineStr">
         <is>
           <t>Supply-chain compliance software for manufacturers, covering product compliance and ESG.</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20" ht="48" customHeight="1">
+      <c r="M19" s="10" t="inlineStr"/>
+    </row>
+    <row r="20" ht="72" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Supplier compliance</t>
@@ -1624,29 +1884,39 @@
           <t>Not confirmed in the sources checked for this list</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Josefin Gullbrandsson, Head of Marketing and Communications.</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
         <is>
           <t>https://www.worldfavor.com</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="K20" s="7" t="inlineStr">
         <is>
           <t>https://blog.worldfavor.com/</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="L20" s="7" t="inlineStr">
         <is>
           <t>Software for collecting supplier sustainability data and producing reports.</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21" ht="48" customHeight="1">
+      <c r="M20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21" ht="72" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Supplier compliance</t>
@@ -1677,33 +1947,43 @@
           <t>Not confirmed in the sources checked for this list</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>Founder — confirm the name on the about page before you email.</t>
+        </is>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
         <is>
           <t>https://www.tennaxia.com</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="K21" s="10" t="inlineStr">
         <is>
           <t>https://www.tennaxia.com/blog</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="L21" s="10" t="inlineStr">
         <is>
           <t>French sustainability-reporting software for measuring impact and running ESG reporting.</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="M21" s="10" t="inlineStr">
         <is>
           <t>A comparison by Sami said Tennaxia acquired Traace. Confirm that before you mention it.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="48" customHeight="1">
+    <row r="22" ht="72" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Traceability</t>
@@ -1734,33 +2014,43 @@
           <t>Douglas Johnson-Poensgen, Veera Johnson</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Douglas Johnson-Poensgen, founder. No current content lead found. The company is small, so budget is the risk.</t>
+        </is>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
         <is>
           <t>https://www.circulor.com</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="K22" s="7" t="inlineStr">
         <is>
           <t>https://www.circulor.com</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="L22" s="7" t="inlineStr">
         <is>
           <t>Traceability software for raw-material supply chains, including batteries and mined materials.</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="M22" s="7" t="inlineStr">
         <is>
           <t>No separate blog URL was confirmed. Use a page from the site in your note.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="48" customHeight="1">
+    <row r="23" ht="72" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Traceability</t>
@@ -1791,33 +2081,43 @@
           <t>Leonardo Bonanni</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Leonardo Bonanni, founder. No current content lead found.</t>
+        </is>
+      </c>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
         <is>
           <t>https://www.sourcemap.com</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="K23" s="10" t="inlineStr">
         <is>
           <t>https://www.sourcemap.com</t>
         </is>
       </c>
-      <c r="J23" s="5" t="inlineStr">
+      <c r="L23" s="10" t="inlineStr">
         <is>
           <t>Supply-chain mapping software for due diligence from raw material to finished product.</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr">
+      <c r="M23" s="10" t="inlineStr">
         <is>
           <t>Also has a presence in France.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="48" customHeight="1">
+    <row r="24" ht="72" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Traceability</t>
@@ -1848,33 +2148,43 @@
           <t>Shameek Ghosh, Hrishikesh Rajan, Madhava Venkatesh, Saravanan Parisutham</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Marketing or content lead — the name was not confirmed. Check LinkedIn before you assume the seat is empty. The team is large enough to have one.</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>https://trustrace.com</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="K24" s="7" t="inlineStr">
         <is>
           <t>https://trustrace.com/our-story</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="L24" s="7" t="inlineStr">
         <is>
           <t>Traceability software for fashion and footwear brands.</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
+      <c r="M24" s="7" t="inlineStr">
         <is>
           <t>The story page is the confirmed content URL. Look for a magazine or blog in the menu.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="48" customHeight="1">
+    <row r="25" ht="72" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Traceability</t>
@@ -1905,29 +2215,39 @@
           <t>Jessi Baker</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>Jessi Baker, founder. No current content lead found.</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J25" s="10" t="inlineStr">
         <is>
           <t>https://www.provenance.org</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="K25" s="10" t="inlineStr">
         <is>
           <t>https://www.provenance.org/news-insights</t>
         </is>
       </c>
-      <c r="J25" s="5" t="inlineStr">
+      <c r="L25" s="10" t="inlineStr">
         <is>
           <t>Product traceability software that lets brands show where a product came from.</t>
         </is>
       </c>
-      <c r="K25" s="5" t="inlineStr"/>
-    </row>
-    <row r="26" ht="48" customHeight="1">
+      <c r="M25" s="10" t="inlineStr"/>
+    </row>
+    <row r="26" ht="72" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Traceability</t>
@@ -1958,33 +2278,43 @@
           <t>Not confirmed in the sources checked for this list</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Marketing lead — the name was not confirmed. Check LinkedIn. The company is large enough that a marketing team is likely.</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="inlineStr">
         <is>
           <t>https://www.optelgroup.com/en/</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="K26" s="7" t="inlineStr">
         <is>
           <t>https://www.optelgroup.com/en/</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="L26" s="7" t="inlineStr">
         <is>
           <t>Track-and-trace and supply-chain software, including carbon tracking and digital product passports.</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="M26" s="7" t="inlineStr">
         <is>
           <t>A blog is linked in the site menu. Confirm the city and the founder on the about page. French is a real pitching language here.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="48" customHeight="1">
+    <row r="27" ht="72" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Traceability</t>
@@ -2015,33 +2345,43 @@
           <t>Not confirmed in the sources checked for this list</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>Isma Chanez, Global Head of Marketing and Product Marketing. The public profile describes a team that includes content.</t>
+        </is>
+      </c>
+      <c r="I27" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J27" s="10" t="inlineStr">
         <is>
           <t>https://www.retraced.com</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="K27" s="10" t="inlineStr">
         <is>
           <t>https://www.retraced.com</t>
         </is>
       </c>
-      <c r="J27" s="5" t="inlineStr">
+      <c r="L27" s="10" t="inlineStr">
         <is>
           <t>Supply-chain transparency and compliance software for fashion and textile brands.</t>
         </is>
       </c>
-      <c r="K27" s="5" t="inlineStr">
+      <c r="M27" s="10" t="inlineStr">
         <is>
           <t>A magazine is linked in the site menu. Confirm the founder before you email.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="48" customHeight="1">
+    <row r="28" ht="72" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Traceability</t>
@@ -2072,33 +2412,43 @@
           <t>Not confirmed in the sources checked for this list</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Do not pitch. Former employer. Public profiles list a senior marketing manager, and headcount has been shrinking.</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="inlineStr">
         <is>
           <t>https://opensc.org</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="K28" s="7" t="inlineStr">
         <is>
           <t>https://opensc.org</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="L28" s="7" t="inlineStr">
         <is>
           <t>Traceability software that verifies sustainable food production at the source.</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="M28" s="7" t="inlineStr">
         <is>
           <t>You used to work here. Do not use Nespresso or other client material without written permission.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="48" customHeight="1">
+    <row r="29" ht="72" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Product carbon, adjacent</t>
@@ -2129,33 +2479,43 @@
           <t>Not confirmed in the sources checked for this list</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>Founder — confirm the name on the site, and confirm whether the brand is Makersite or Mattermaps.</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
         <is>
           <t>https://makersite.io</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="K29" s="10" t="inlineStr">
         <is>
           <t>https://makersite.io</t>
         </is>
       </c>
-      <c r="J29" s="5" t="inlineStr">
+      <c r="L29" s="10" t="inlineStr">
         <is>
           <t>Software for product life-cycle data, product carbon footprints, and supply-chain emissions.</t>
         </is>
       </c>
-      <c r="K29" s="5" t="inlineStr">
+      <c r="M29" s="10" t="inlineStr">
         <is>
           <t>The site has used both the Makersite and Mattermaps names. Confirm the current brand and city.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="48" customHeight="1">
+    <row r="30" ht="72" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>ESG reporting, adjacent</t>
@@ -2186,34 +2546,44 @@
           <t>Not confirmed in the sources checked for this list</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>Not publicly listed</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Founder — confirm the name on the about page. This is ESG reporting software, adjacent to the niche.</t>
+        </is>
+      </c>
+      <c r="I30" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J30" s="7" t="inlineStr">
         <is>
           <t>https://novisto.com</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="K30" s="7" t="inlineStr">
         <is>
           <t>https://novisto.com</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="L30" s="7" t="inlineStr">
         <is>
           <t>ESG data collection and reporting software. Adjacent to supplier climate work, not a traceability tool.</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
+      <c r="M30" s="7" t="inlineStr">
         <is>
           <t>No separate blog URL was confirmed.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K30"/>
+  <autoFilter ref="A1:M30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add CAA conference organisations to the target list.
Include speakers, programme names, biography affiliations, the participant-list firms, and the extra organisations Nicolas named. Climatiq and Sami stay on their existing rows.

Co-authored-by: nicolasmpicard-gif <nicolasmpicard-gif@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Supply-chain-climate-company-targets.xlsx
+++ b/Supply-chain-climate-company-targets.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Companies" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Companies'!$A$1:$M$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Companies'!$A$1:$M$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -60,7 +60,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -95,6 +95,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FBF3D5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7EEF8"/>
       </patternFill>
     </fill>
   </fills>
@@ -138,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -172,6 +177,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -552,7 +560,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="280" customHeight="1">
+    <row r="2" ht="360" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>This is a working target list, not a census of every company in the world. It covers firms that sell supplier compliance, traceability, or carbon-data software and that publish in English or French. Plan A, Cozero, Climatiq, Vaayu, and carbmee are included.
@@ -563,7 +571,8 @@
 Where a founder could not be confirmed from a page opened for this list, the cell says so. Do not guess. Open the about page and fill the name yourself.
 Use the Content page column to find one specific article, then mention that article in the email and propose one title.
 IntegrityNext and OpenSC are former employers. Do not attach or describe confidential client work.
-Filter the Probability column. Start with High, in carbon data and supplier compliance, in France, the UK, and Berlin. Traceability is the same buyer only when the product is about proof of origin or supplier data.</t>
+Filter the Probability column. Start with High, in carbon data and supplier compliance, in France, the UK, and Berlin. Traceability is the same buyer only when the product is about proof of origin or supplier data.
+Rows marked CAA 2026 were added from the conference agenda, the speakers page, and the agenda PDF for 6 October 2026 in London, plus organisations Nicolas identified on the participant list. Rows marked Added by you are the extra organisations he named. Own content? is Not checked and Probability is Not scored on all of those rows, because content staffing was not researched. Confirm the person still works there before you email. Climatiq and Sami were already on this list. Their rows note that they are on the programme. Do not add them again. A biography row is a past role or a side affiliation. Do not email that organisation as if the speaker still works there.</t>
         </is>
       </c>
     </row>
@@ -578,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:M97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -854,7 +863,11 @@
           <t>Emission-factor data and carbon calculation tools that other software can plug into.</t>
         </is>
       </c>
-      <c r="M4" s="7" t="inlineStr"/>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>Hessam Lavi, CEO and co-founder, is speaking at the CAA conference in London on 6 October 2026, including the PCF clinic. The content contact is still Madeleine Ralph.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -1215,7 +1228,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Not confirmed in the sources checked for this list</t>
+          <t>Tanguy Robert (co-founder, named on the CAA 2026 speakers page). Any other founders were not confirmed.</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1250,7 +1263,7 @@
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>SGS took a majority stake in November 2025. Find the founder on the company site before you email.</t>
+          <t>SGS took a majority stake in November 2025. Tanguy Robert is speaking on AI and carbon accounting at the CAA conference in London on 6 October 2026. Confirm marketing spend is still open before you email.</t>
         </is>
       </c>
     </row>
@@ -2582,8 +2595,4497 @@
         </is>
       </c>
     </row>
+    <row r="31" ht="78" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>ALDI South Group</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>English and German</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>KT Michaelson, Global Director, Climate and Nature. Erik Björke, Global Manager for Environmental Data and Risks, ALDI SÜD HOLDING, is on a later panel.</t>
+        </is>
+      </c>
+      <c r="I31" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aldi-sued.com</t>
+        </is>
+      </c>
+      <c r="K31" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aldi-sued.com</t>
+        </is>
+      </c>
+      <c r="L31" s="9" t="inlineStr">
+        <is>
+          <t>International retail group. Two of its sustainability leaders are on the CAA programme.</t>
+        </is>
+      </c>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>The agenda uses both The ALDI South Group and ALDI SÜD HOLDING. Confirm which entity you are writing to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="78" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Anthesis</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Do not email Jono Adams as a current employee. The agenda lists him as Exec Director for Climate, Ex-Anthesis, moderating as an independent.</t>
+        </is>
+      </c>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>https://www.anthesisgroup.com</t>
+        </is>
+      </c>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>https://www.anthesisgroup.com</t>
+        </is>
+      </c>
+      <c r="L32" s="7" t="inlineStr">
+        <is>
+          <t>Sustainability consultancy named because a former executive is moderating a CAA session.</t>
+        </is>
+      </c>
+      <c r="M32" s="7" t="inlineStr">
+        <is>
+          <t>Find a current Anthesis contact on the site. Jono Adams is listed as ex-Anthesis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="78" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Carbon Accounting Alliance</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Andrew Griffiths and Emilien Hoet</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H33" s="9" t="inlineStr">
+        <is>
+          <t>Andrew Griffiths and Emilien Hoet, co-founders. They open, host, and close the 6 October 2026 conference.</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J33" s="9" t="inlineStr">
+        <is>
+          <t>https://www.carbonaccountingalliance.com</t>
+        </is>
+      </c>
+      <c r="K33" s="9" t="inlineStr">
+        <is>
+          <t>https://conference.carbonaccountingalliance.com/agenda-2026</t>
+        </is>
+      </c>
+      <c r="L33" s="9" t="inlineStr">
+        <is>
+          <t>Membership alliance for carbon-accounting practitioners. Host of the London conference on 6 October 2026.</t>
+        </is>
+      </c>
+      <c r="M33" s="9" t="inlineStr">
+        <is>
+          <t>The agenda also mentions the RCAA professional register. Treat that as a CAA initiative, not a separate company, until you confirm otherwise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="78" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Carbon Data Open Protocol</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed. Shona Crawford-Smith of Sylvera is a co-chair.</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Shona Crawford-Smith, General Manager at Sylvera and a CDOP co-chair.</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>https://www.cdop.info</t>
+        </is>
+      </c>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>https://www.cdop.info</t>
+        </is>
+      </c>
+      <c r="L34" s="7" t="inlineStr">
+        <is>
+          <t>Cross-industry effort to standardise data about carbon-crediting projects and carbon credits.</t>
+        </is>
+      </c>
+      <c r="M34" s="7" t="inlineStr">
+        <is>
+          <t>CDOP’s own FAQ says it is co-chaired by organisations, including Sylvera. Write to Shona about Sylvera or about CDOP, and say which.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="78" customHeight="1">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Carbonology</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>Melanie Blackmore</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>Melanie Blackmore, CEO and founder.</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J35" s="9" t="inlineStr">
+        <is>
+          <t>https://www.carbonologyverification.com</t>
+        </is>
+      </c>
+      <c r="K35" s="9" t="inlineStr">
+        <is>
+          <t>https://www.carbonologyverification.com/about-us</t>
+        </is>
+      </c>
+      <c r="L35" s="9" t="inlineStr">
+        <is>
+          <t>UK verification body for greenhouse-gas statements, including ISO 14064.</t>
+        </is>
+      </c>
+      <c r="M35" s="9" t="inlineStr">
+        <is>
+          <t>Listed as a CAA roundtable moderator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="78" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>CDP</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Paul Dickinson</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Paul Dickinson, founder. He is also co-founder of Transition Value Partners.</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="inlineStr">
+        <is>
+          <t>https://www.cdp.net</t>
+        </is>
+      </c>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>https://www.cdp.net</t>
+        </is>
+      </c>
+      <c r="L36" s="7" t="inlineStr">
+        <is>
+          <t>Global disclosure system for companies, cities, and public authorities to report environmental impact.</t>
+        </is>
+      </c>
+      <c r="M36" s="7" t="inlineStr">
+        <is>
+          <t>Paul is on the net-zero panel. Confirm he is the right CDP contact, rather than the current executive team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="78" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Center for Green Market Activation</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H37" s="9" t="inlineStr">
+        <is>
+          <t>Laura Draucker, Standards and Guidance Director. She also chairs the SBTi Technical Council.</t>
+        </is>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J37" s="9" t="inlineStr">
+        <is>
+          <t>https://gmacenter.org</t>
+        </is>
+      </c>
+      <c r="K37" s="9" t="inlineStr">
+        <is>
+          <t>https://gmacenter.org/programs/</t>
+        </is>
+      </c>
+      <c r="L37" s="9" t="inlineStr">
+        <is>
+          <t>US nonprofit that aggregates demand for low-carbon fuels and materials, including through the AIM Platform.</t>
+        </is>
+      </c>
+      <c r="M37" s="9" t="inlineStr">
+        <is>
+          <t>The agenda abbreviates the name as Center for GMA. The speakers page spells out Center for Green Market Activation. AIM Platform is a partnership with C2ES and Gold Standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="78" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>ClimatePartner</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>English and German</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Andrew Pridding, Head of Delivery, and Daniela Contreras, Project Manager and Senior Sustainability Consultant.</t>
+        </is>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>https://www.climatepartner.com</t>
+        </is>
+      </c>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>https://www.climatepartner.com</t>
+        </is>
+      </c>
+      <c r="L38" s="7" t="inlineStr">
+        <is>
+          <t>Climate-action and carbon-management consultancy. Two of its people are CAA roundtable moderators.</t>
+        </is>
+      </c>
+      <c r="M38" s="7" t="inlineStr">
+        <is>
+          <t>Listed on the CAA speakers page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="78" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>ECOS</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Brussels</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>Thea Lyngseth, Programme Officer, Carbon Accounting and Management.</t>
+        </is>
+      </c>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J39" s="9" t="inlineStr">
+        <is>
+          <t>https://ecostandard.org</t>
+        </is>
+      </c>
+      <c r="K39" s="9" t="inlineStr">
+        <is>
+          <t>https://ecostandard.org</t>
+        </is>
+      </c>
+      <c r="L39" s="9" t="inlineStr">
+        <is>
+          <t>Network of environmental NGOs that works on standards and product rules, including GHG accounting and net zero.</t>
+        </is>
+      </c>
+      <c r="M39" s="9" t="inlineStr">
+        <is>
+          <t>Listed as a CAA roundtable moderator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="78" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>EnergyTag</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Ellie Rowlands, Communications Manager.</t>
+        </is>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>https://energytag.org</t>
+        </is>
+      </c>
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t>https://energytag.org</t>
+        </is>
+      </c>
+      <c r="L40" s="7" t="inlineStr">
+        <is>
+          <t>Organisation working on hourly, more granular renewable-energy certificates.</t>
+        </is>
+      </c>
+      <c r="M40" s="7" t="inlineStr">
+        <is>
+          <t>Listed as a CAA roundtable moderator. Ellie previously worked at Energy UK, Ripple Energy, and Rebel Energy. Those are past roles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="78" customHeight="1">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Forum for the Future</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>Jonathon Porritt (co-founder)</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H41" s="9" t="inlineStr">
+        <is>
+          <t>Jonathon Porritt, founder, giving the morning keynote.</t>
+        </is>
+      </c>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J41" s="9" t="inlineStr">
+        <is>
+          <t>https://www.forumforthefuture.org</t>
+        </is>
+      </c>
+      <c r="K41" s="9" t="inlineStr">
+        <is>
+          <t>https://www.forumforthefuture.org</t>
+        </is>
+      </c>
+      <c r="L41" s="9" t="inlineStr">
+        <is>
+          <t>International sustainability nonprofit. Jonathon Porritt co-founded it in 1996.</t>
+        </is>
+      </c>
+      <c r="M41" s="9" t="inlineStr">
+        <is>
+          <t>Keynote speaker at the CAA conference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="78" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>GHG Protocol</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Tim Mohin, CEO.</t>
+        </is>
+      </c>
+      <c r="I42" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>https://ghgprotocol.org</t>
+        </is>
+      </c>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>https://ghgprotocol.org</t>
+        </is>
+      </c>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
+          <t>The greenhouse-gas accounting standards used by companies worldwide. Tim Mohin is in conversation with the CAA co-founder.</t>
+        </is>
+      </c>
+      <c r="M42" s="7" t="inlineStr">
+        <is>
+          <t>The agenda says the Protocol is updating its standards and working on a merger with ISO. Tim previously led the Global Reporting Initiative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="78" customHeight="1">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>ISEP</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Lincoln</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>Not a founder-led company. It is a professional body.</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>Sue Buxey, Director of Operations and Professional Standards. Chloë Fiddy, Senior Policy and Engagement Lead, is a roundtable moderator.</t>
+        </is>
+      </c>
+      <c r="I43" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J43" s="9" t="inlineStr">
+        <is>
+          <t>https://www.isepglobal.org</t>
+        </is>
+      </c>
+      <c r="K43" s="9" t="inlineStr">
+        <is>
+          <t>https://www.isepglobal.org</t>
+        </is>
+      </c>
+      <c r="L43" s="9" t="inlineStr">
+        <is>
+          <t>Institute of Sustainability and Environmental Professionals, formerly IEMA. The morning includes a partnership announcement with the CAA.</t>
+        </is>
+      </c>
+      <c r="M43" s="9" t="inlineStr">
+        <is>
+          <t>Two ISEP staff are on the programme. Sue also sits on the board of the Society for the Environment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="78" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Logitech</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Lausanne</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Caroline Kennedy, Director and Head of Climate, Circularity and Reporting.</t>
+        </is>
+      </c>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J44" s="7" t="inlineStr">
+        <is>
+          <t>https://www.logitech.com</t>
+        </is>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>https://www.logitech.com</t>
+        </is>
+      </c>
+      <c r="L44" s="7" t="inlineStr">
+        <is>
+          <t>Electronics company. Caroline leads climate, circularity, and reporting, including product carbon footprints.</t>
+        </is>
+      </c>
+      <c r="M44" s="7" t="inlineStr">
+        <is>
+          <t>On the PCF session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="78" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Mars Inc.</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>McLean</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>Ian Knight, Global Sustainability Director.</t>
+        </is>
+      </c>
+      <c r="I45" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J45" s="9" t="inlineStr">
+        <is>
+          <t>https://www.mars.com</t>
+        </is>
+      </c>
+      <c r="K45" s="9" t="inlineStr">
+        <is>
+          <t>https://www.mars.com</t>
+        </is>
+      </c>
+      <c r="L45" s="9" t="inlineStr">
+        <is>
+          <t>Food company. Ian covers renewable energy, environmental attribute certificates, and factory and logistics sustainability.</t>
+        </is>
+      </c>
+      <c r="M45" s="9" t="inlineStr">
+        <is>
+          <t>On the Scope 3 panel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="78" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>NHS England</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>Not a founder-led company.</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Alexandra Hammond, Associate Director, Net Zero and Sustainable Procurement.</t>
+        </is>
+      </c>
+      <c r="I46" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J46" s="7" t="inlineStr">
+        <is>
+          <t>https://www.england.nhs.uk</t>
+        </is>
+      </c>
+      <c r="K46" s="7" t="inlineStr">
+        <is>
+          <t>https://www.england.nhs.uk</t>
+        </is>
+      </c>
+      <c r="L46" s="7" t="inlineStr">
+        <is>
+          <t>National health body. Alexandra leads supplier decarbonisation for one of the largest healthcare supply chains.</t>
+        </is>
+      </c>
+      <c r="M46" s="7" t="inlineStr">
+        <is>
+          <t>On the Scope 3 panel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="78" customHeight="1">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>Oxford Net Zero</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Oxford</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>Kaya Axelsson, Director of Impact.</t>
+        </is>
+      </c>
+      <c r="I47" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J47" s="9" t="inlineStr">
+        <is>
+          <t>https://netzeroclimate.org</t>
+        </is>
+      </c>
+      <c r="K47" s="9" t="inlineStr">
+        <is>
+          <t>https://netzeroclimate.org</t>
+        </is>
+      </c>
+      <c r="L47" s="9" t="inlineStr">
+        <is>
+          <t>University of Oxford programme on net-zero governance and practice.</t>
+        </is>
+      </c>
+      <c r="M47" s="9" t="inlineStr">
+        <is>
+          <t>On the net-zero panel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="78" customHeight="1">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Rawstone Consulting</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Caroline Johnstone</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>Caroline Johnstone, founder and Managing Director.</t>
+        </is>
+      </c>
+      <c r="I48" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>https://www.rawstoneconsulting.co.uk</t>
+        </is>
+      </c>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>https://www.rawstoneconsulting.co.uk/about</t>
+        </is>
+      </c>
+      <c r="L48" s="7" t="inlineStr">
+        <is>
+          <t>ESG and greenhouse-gas consultancy for medium and large organisations. Founded in 2018.</t>
+        </is>
+      </c>
+      <c r="M48" s="7" t="inlineStr">
+        <is>
+          <t>Listed as a CAA roundtable moderator. The about page says she is a member of the Carbon Accounting Alliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="78" customHeight="1">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>Sandoz</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>Basel</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="inlineStr">
+        <is>
+          <t>Ben Thornton-Jones, Head of Procurement ESG.</t>
+        </is>
+      </c>
+      <c r="I49" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J49" s="9" t="inlineStr">
+        <is>
+          <t>https://www.sandoz.com</t>
+        </is>
+      </c>
+      <c r="K49" s="9" t="inlineStr">
+        <is>
+          <t>https://www.sandoz.com</t>
+        </is>
+      </c>
+      <c r="L49" s="9" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals company. Ben leads procurement ESG.</t>
+        </is>
+      </c>
+      <c r="M49" s="9" t="inlineStr">
+        <is>
+          <t>On the Scope 3 panel. He previously worked at Haleon and GSK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="78" customHeight="1">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Scope 3 Peer Group</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>Oliver Hurrey</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>Oliver Hurrey, founder and chair. He moderates two sessions.</t>
+        </is>
+      </c>
+      <c r="I50" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>https://www.scope3peergroup.com</t>
+        </is>
+      </c>
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t>https://www.scope3peergroup.com</t>
+        </is>
+      </c>
+      <c r="L50" s="7" t="inlineStr">
+        <is>
+          <t>Peer group of practitioners working on supply-chain emissions. Its logo is on the PCF clinic as a collaborator.</t>
+        </is>
+      </c>
+      <c r="M50" s="7" t="inlineStr">
+        <is>
+          <t>Oliver is also a steering-group member of the Sustainable Procurement Pledge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="78" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>Small World Consulting</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Mike Berners-Lee</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>Mike Berners-Lee, founder. The agenda gives him an announcement slot, and he is a roundtable moderator.</t>
+        </is>
+      </c>
+      <c r="I51" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J51" s="9" t="inlineStr">
+        <is>
+          <t>https://www.sw-consulting.co.uk</t>
+        </is>
+      </c>
+      <c r="K51" s="9" t="inlineStr">
+        <is>
+          <t>https://www.sw-consulting.co.uk</t>
+        </is>
+      </c>
+      <c r="L51" s="9" t="inlineStr">
+        <is>
+          <t>Carbon and sustainability consultancy led by Mike Berners-Lee.</t>
+        </is>
+      </c>
+      <c r="M51" s="9" t="inlineStr">
+        <is>
+          <t>He is also a professor at Lancaster University. That is a separate academic role.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="78" customHeight="1">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Sustainable AI Group</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>Boris Gamazaychikov (co-founder and CEO). Other co-founders were not confirmed here.</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>Boris Gamazaychikov, co-founder and CEO.</t>
+        </is>
+      </c>
+      <c r="I52" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J52" s="7" t="inlineStr">
+        <is>
+          <t>https://sustainableaigroup.com</t>
+        </is>
+      </c>
+      <c r="K52" s="7" t="inlineStr">
+        <is>
+          <t>https://sustainableaigroup.com</t>
+        </is>
+      </c>
+      <c r="L52" s="7" t="inlineStr">
+        <is>
+          <t>Research and advisory firm on the environmental impact of AI.</t>
+        </is>
+      </c>
+      <c r="M52" s="7" t="inlineStr">
+        <is>
+          <t>On the AI and carbon-accounting session. He previously led AI sustainability at Salesforce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="78" customHeight="1">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>Sustainable Procurement Pledge</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H53" s="9" t="inlineStr">
+        <is>
+          <t>Oliver Hurrey sits on the steering group. His main listed role is founder of the Scope 3 Peer Group.</t>
+        </is>
+      </c>
+      <c r="I53" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J53" s="9" t="inlineStr">
+        <is>
+          <t>https://www.spp.earth</t>
+        </is>
+      </c>
+      <c r="K53" s="9" t="inlineStr">
+        <is>
+          <t>https://www.spp.earth</t>
+        </is>
+      </c>
+      <c r="L53" s="9" t="inlineStr">
+        <is>
+          <t>Pledge aimed at getting procurement professionals to build sustainability into how they buy.</t>
+        </is>
+      </c>
+      <c r="M53" s="9" t="inlineStr">
+        <is>
+          <t>Named in Oliver Hurrey’s speaker biography, not as his job title.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="78" customHeight="1">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Sylvera</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>Shona Crawford-Smith, General Manager. She co-chairs the Carbon Data Open Protocol.</t>
+        </is>
+      </c>
+      <c r="I54" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J54" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sylvera.com</t>
+        </is>
+      </c>
+      <c r="K54" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sylvera.com</t>
+        </is>
+      </c>
+      <c r="L54" s="7" t="inlineStr">
+        <is>
+          <t>Carbon-market data and ratings company. Shona leads the carbon-differentiated commodities business.</t>
+        </is>
+      </c>
+      <c r="M54" s="7" t="inlineStr">
+        <is>
+          <t>Listed as a CAA roundtable moderator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="78" customHeight="1">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>Symbiosis Leadership</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>Alexander Schmidt</t>
+        </is>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>Dr Alexander Schmidt, founder.</t>
+        </is>
+      </c>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J55" s="9" t="inlineStr">
+        <is>
+          <t>https://symbiosisleadership.com</t>
+        </is>
+      </c>
+      <c r="K55" s="9" t="inlineStr">
+        <is>
+          <t>https://symbiosisleadership.com</t>
+        </is>
+      </c>
+      <c r="L55" s="9" t="inlineStr">
+        <is>
+          <t>Convening practice for leaders working on problems that cut across organisations. He also contributes to climate-accountability standards.</t>
+        </is>
+      </c>
+      <c r="M55" s="9" t="inlineStr">
+        <is>
+          <t>Listed as a CAA roundtable moderator. He is a Fellow of the Exponential Roadmap Initiative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="78" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Syntegon</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Waiblingen</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>English and German</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>Stella Constantatos, Director, Climate and Environment.</t>
+        </is>
+      </c>
+      <c r="I56" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>https://www.syntegon.com</t>
+        </is>
+      </c>
+      <c r="K56" s="7" t="inlineStr">
+        <is>
+          <t>https://www.syntegon.com</t>
+        </is>
+      </c>
+      <c r="L56" s="7" t="inlineStr">
+        <is>
+          <t>Processing and packaging technology company. Stella leads climate and environment.</t>
+        </is>
+      </c>
+      <c r="M56" s="7" t="inlineStr">
+        <is>
+          <t>Listed as a CAA roundtable moderator. She previously led Unilever’s Supplier Climate Programme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="78" customHeight="1">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>The Climate Source</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>Orland</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="inlineStr">
+        <is>
+          <t>Jessie Deelo (co-founder and CEO). Other co-founders were not confirmed here.</t>
+        </is>
+      </c>
+      <c r="G57" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H57" s="9" t="inlineStr">
+        <is>
+          <t>Jessie Deelo, CEO and co-founder.</t>
+        </is>
+      </c>
+      <c r="I57" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J57" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="K57" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="L57" s="9" t="inlineStr">
+        <is>
+          <t>Designs market-based strategies for agricultural supply chains, including the BoundDairy carbon-accounting platform.</t>
+        </is>
+      </c>
+      <c r="M57" s="9" t="inlineStr">
+        <is>
+          <t>City is from a public profile and should be confirmed. No company website was confirmed in this pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="78" customHeight="1">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Thrive Accountants</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>East Grinstead</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>James Lizars</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>James Lizars, founder.</t>
+        </is>
+      </c>
+      <c r="I58" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>https://thrive.accountants</t>
+        </is>
+      </c>
+      <c r="K58" s="7" t="inlineStr">
+        <is>
+          <t>https://thrive.accountants</t>
+        </is>
+      </c>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t>B Corp accountancy firm for early-stage tech founders. James is on the panel about professionalising carbon accounting.</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="inlineStr">
+        <is>
+          <t>Listed on the CAA programme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="78" customHeight="1">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>Transition Value Partners</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="E59" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="inlineStr">
+        <is>
+          <t>Paul Dickinson (co-founder). Other co-founders were not confirmed here.</t>
+        </is>
+      </c>
+      <c r="G59" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H59" s="9" t="inlineStr">
+        <is>
+          <t>Paul Dickinson, co-founder. His speaker title also lists him as founder of CDP.</t>
+        </is>
+      </c>
+      <c r="I59" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J59" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="K59" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="L59" s="9" t="inlineStr">
+        <is>
+          <t>Firm co-founded by Paul Dickinson, who is on the CAA net-zero panel.</t>
+        </is>
+      </c>
+      <c r="M59" s="9" t="inlineStr">
+        <is>
+          <t>No public website was confirmed in this pass. Do not guess the URL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="78" customHeight="1">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>UK Carbon Verification</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Guildford</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>Matt Letley</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H60" s="7" t="inlineStr">
+        <is>
+          <t>Matt Letley, founder and CEO. He was previously Commercial Director at Planet Mark.</t>
+        </is>
+      </c>
+      <c r="I60" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J60" s="7" t="inlineStr">
+        <is>
+          <t>https://www.ukcarbonverification.com</t>
+        </is>
+      </c>
+      <c r="K60" s="7" t="inlineStr">
+        <is>
+          <t>https://www.ukcarbonverification.com</t>
+        </is>
+      </c>
+      <c r="L60" s="7" t="inlineStr">
+        <is>
+          <t>Independent verification and assurance firm for organisational greenhouse-gas inventories. Founded in 2026.</t>
+        </is>
+      </c>
+      <c r="M60" s="7" t="inlineStr">
+        <is>
+          <t>Listed as a CAA roundtable moderator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="78" customHeight="1">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="inlineStr">
+        <is>
+          <t>Unilever</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D61" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E61" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G61" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H61" s="9" t="inlineStr">
+        <is>
+          <t>Dr Katy Armstrong, Environmental Sustainability Scientist.</t>
+        </is>
+      </c>
+      <c r="I61" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J61" s="9" t="inlineStr">
+        <is>
+          <t>https://www.unilever.com</t>
+        </is>
+      </c>
+      <c r="K61" s="9" t="inlineStr">
+        <is>
+          <t>https://www.unilever.com</t>
+        </is>
+      </c>
+      <c r="L61" s="9" t="inlineStr">
+        <is>
+          <t>Consumer-goods company. Katy leads environmental assessments for new technologies, ingredients, and products, and sits on the PACT methodology group.</t>
+        </is>
+      </c>
+      <c r="M61" s="9" t="inlineStr">
+        <is>
+          <t>On the PCF clinic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="78" customHeight="1">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>University of Edinburgh</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Edinburgh</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>Not a founder-led company.</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>Matthew Brander, Chair of Carbon Accounting, and Dr Michelle O’Keeffe, Senior Research Fellow, both at the University of Edinburgh Business School.</t>
+        </is>
+      </c>
+      <c r="I62" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>https://www.business-school.ed.ac.uk</t>
+        </is>
+      </c>
+      <c r="K62" s="7" t="inlineStr">
+        <is>
+          <t>https://www.business-school.ed.ac.uk</t>
+        </is>
+      </c>
+      <c r="L62" s="7" t="inlineStr">
+        <is>
+          <t>Matthew holds the Chair of Carbon Accounting and is speaking on which accounting method fits which decision.</t>
+        </is>
+      </c>
+      <c r="M62" s="7" t="inlineStr">
+        <is>
+          <t>Academic speakers, not a software vendor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="78" customHeight="1">
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B63" s="9" t="inlineStr">
+        <is>
+          <t>vybcheck</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D63" s="9" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E63" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="inlineStr">
+        <is>
+          <t>Beth Thayne and Ross Bermudez</t>
+        </is>
+      </c>
+      <c r="G63" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H63" s="9" t="inlineStr">
+        <is>
+          <t>Beth Thayne, co-founder. She is moderating the AI session.</t>
+        </is>
+      </c>
+      <c r="I63" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J63" s="9" t="inlineStr">
+        <is>
+          <t>https://vybcheck.it.com</t>
+        </is>
+      </c>
+      <c r="K63" s="9" t="inlineStr">
+        <is>
+          <t>https://vybcheck.it.com</t>
+        </is>
+      </c>
+      <c r="L63" s="9" t="inlineStr">
+        <is>
+          <t>Small practice on building with AI, from technical setup to team training.</t>
+        </is>
+      </c>
+      <c r="M63" s="9" t="inlineStr">
+        <is>
+          <t>A public profile lists the homepage as vybcheck.it.com and the team as based in Germany. Confirm both before you email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="78" customHeight="1">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>WBCSD</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Geneva</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H64" s="7" t="inlineStr">
+        <is>
+          <t>Izzy Farnsworth, Senior Associate for PACT. Inês Amorim, Manager, Climate Action, and Kalina Paprzycka, Climate Action Associate, are roundtable moderators.</t>
+        </is>
+      </c>
+      <c r="I64" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t>https://www.wbcsd.org</t>
+        </is>
+      </c>
+      <c r="K64" s="7" t="inlineStr">
+        <is>
+          <t>https://www.wbcsd.org</t>
+        </is>
+      </c>
+      <c r="L64" s="7" t="inlineStr">
+        <is>
+          <t>World Business Council for Sustainable Development. PACT, its product-carbon-footprint data exchange, is a collaborator on the PCF clinic.</t>
+        </is>
+      </c>
+      <c r="M64" s="7" t="inlineStr">
+        <is>
+          <t>The agenda spells the PACT speaker Izzy Farnsworth. The speakers page spells the name Isobel Farnsworth. Same person.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="78" customHeight="1">
+      <c r="A65" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B65" s="9" t="inlineStr">
+        <is>
+          <t>WRAP</t>
+        </is>
+      </c>
+      <c r="C65" s="9" t="inlineStr">
+        <is>
+          <t>Banbury</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E65" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G65" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H65" s="9" t="inlineStr">
+        <is>
+          <t>Hamish Forbes, Specialist, Food System GHGs.</t>
+        </is>
+      </c>
+      <c r="I65" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J65" s="9" t="inlineStr">
+        <is>
+          <t>https://www.wrap.ngo</t>
+        </is>
+      </c>
+      <c r="K65" s="9" t="inlineStr">
+        <is>
+          <t>https://www.wrap.ngo</t>
+        </is>
+      </c>
+      <c r="L65" s="9" t="inlineStr">
+        <is>
+          <t>UK climate and resources charity. Hamish is on the PCF clinic.</t>
+        </is>
+      </c>
+      <c r="M65" s="9" t="inlineStr">
+        <is>
+          <t>Listed on the CAA agenda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="78" customHeight="1">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — speaker organisation</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Xero</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Wellington</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G66" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H66" s="7" t="inlineStr">
+        <is>
+          <t>Tamara Somers, General Manager, Sustainability and Impact.</t>
+        </is>
+      </c>
+      <c r="I66" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J66" s="7" t="inlineStr">
+        <is>
+          <t>https://www.xero.com</t>
+        </is>
+      </c>
+      <c r="K66" s="7" t="inlineStr">
+        <is>
+          <t>https://www.xero.com</t>
+        </is>
+      </c>
+      <c r="L66" s="7" t="inlineStr">
+        <is>
+          <t>Accounting software company. Tamara leads sustainability and impact and is moderating the professionalisation panel.</t>
+        </is>
+      </c>
+      <c r="M66" s="7" t="inlineStr">
+        <is>
+          <t>Listed on the CAA programme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="78" customHeight="1">
+      <c r="A67" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in the programme</t>
+        </is>
+      </c>
+      <c r="B67" s="9" t="inlineStr">
+        <is>
+          <t>Carbon Measures</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E67" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G67" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H67" s="9" t="inlineStr">
+        <is>
+          <t>No speaker is listed. The net-zero panel description names Carbon Measures as an industry-backed advocacy group.</t>
+        </is>
+      </c>
+      <c r="I67" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J67" s="9" t="inlineStr">
+        <is>
+          <t>https://www.carbonmeasures.org</t>
+        </is>
+      </c>
+      <c r="K67" s="9" t="inlineStr">
+        <is>
+          <t>https://www.carbonmeasures.org</t>
+        </is>
+      </c>
+      <c r="L67" s="9" t="inlineStr">
+        <is>
+          <t>Coalition working on a product-level carbon-accounting framework and product carbon-intensity standards.</t>
+        </is>
+      </c>
+      <c r="M67" s="9" t="inlineStr">
+        <is>
+          <t>Named in the agenda text, not as a speaker’s employer. Find a contact on the site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="78" customHeight="1">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in the programme</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>ISO</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Geneva</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>English and French</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>Not a founder-led company.</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H68" s="7" t="inlineStr">
+        <is>
+          <t>No speaker is listed from ISO. The agenda discusses the ISO Net Zero Standard and a GHG Protocol merger with ISO.</t>
+        </is>
+      </c>
+      <c r="I68" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J68" s="7" t="inlineStr">
+        <is>
+          <t>https://www.iso.org</t>
+        </is>
+      </c>
+      <c r="K68" s="7" t="inlineStr">
+        <is>
+          <t>https://www.iso.org</t>
+        </is>
+      </c>
+      <c r="L68" s="7" t="inlineStr">
+        <is>
+          <t>International standards body. The agenda treats its net-zero work as part of the day’s context.</t>
+        </is>
+      </c>
+      <c r="M68" s="7" t="inlineStr">
+        <is>
+          <t>Named in the programme, not as a speaker’s employer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="78" customHeight="1">
+      <c r="A69" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in the programme</t>
+        </is>
+      </c>
+      <c r="B69" s="9" t="inlineStr">
+        <is>
+          <t>SBTi</t>
+        </is>
+      </c>
+      <c r="C69" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="E69" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G69" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H69" s="9" t="inlineStr">
+        <is>
+          <t>Laura Draucker chairs the SBTi Technical Council. Her speaking role is at the Center for Green Market Activation.</t>
+        </is>
+      </c>
+      <c r="I69" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J69" s="9" t="inlineStr">
+        <is>
+          <t>https://sciencebasedtargets.org</t>
+        </is>
+      </c>
+      <c r="K69" s="9" t="inlineStr">
+        <is>
+          <t>https://sciencebasedtargets.org</t>
+        </is>
+      </c>
+      <c r="L69" s="9" t="inlineStr">
+        <is>
+          <t>Science Based Targets initiative. The net-zero panel is framed around its Net Zero Standard.</t>
+        </is>
+      </c>
+      <c r="M69" s="9" t="inlineStr">
+        <is>
+          <t>Named throughout the agenda. Laura’s employer on the speakers page is GMA, not SBTi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="78" customHeight="1">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in a speaker bio</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Ceres</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>No current speaker. Laura Draucker previously worked there.</t>
+        </is>
+      </c>
+      <c r="I70" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J70" s="7" t="inlineStr">
+        <is>
+          <t>https://www.ceres.org</t>
+        </is>
+      </c>
+      <c r="K70" s="7" t="inlineStr">
+        <is>
+          <t>https://www.ceres.org</t>
+        </is>
+      </c>
+      <c r="L70" s="7" t="inlineStr">
+        <is>
+          <t>Nonprofit that works with investors and companies on sustainability. Named in Laura Draucker’s biography.</t>
+        </is>
+      </c>
+      <c r="M70" s="7" t="inlineStr">
+        <is>
+          <t>Past employer. Do not email as if Laura still works there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="78" customHeight="1">
+      <c r="A71" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in a speaker bio</t>
+        </is>
+      </c>
+      <c r="B71" s="9" t="inlineStr">
+        <is>
+          <t>Energy UK</t>
+        </is>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="inlineStr">
+        <is>
+          <t>Not a founder-led company.</t>
+        </is>
+      </c>
+      <c r="G71" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H71" s="9" t="inlineStr">
+        <is>
+          <t>No current speaker. Ellie Rowlands previously managed stakeholder relationships there.</t>
+        </is>
+      </c>
+      <c r="I71" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J71" s="9" t="inlineStr">
+        <is>
+          <t>https://www.energy-uk.org.uk</t>
+        </is>
+      </c>
+      <c r="K71" s="9" t="inlineStr">
+        <is>
+          <t>https://www.energy-uk.org.uk</t>
+        </is>
+      </c>
+      <c r="L71" s="9" t="inlineStr">
+        <is>
+          <t>Trade association for the UK energy industry. Named in Ellie Rowlands’s biography.</t>
+        </is>
+      </c>
+      <c r="M71" s="9" t="inlineStr">
+        <is>
+          <t>Past employer. Her current role is Communications Manager at EnergyTag.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="78" customHeight="1">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in a speaker bio</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Exponential Roadmap Initiative</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr">
+        <is>
+          <t>Alexander Schmidt is a Fellow. His speaking role is as founder of Symbiosis Leadership.</t>
+        </is>
+      </c>
+      <c r="I72" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J72" s="7" t="inlineStr">
+        <is>
+          <t>https://exponentialroadmap.org</t>
+        </is>
+      </c>
+      <c r="K72" s="7" t="inlineStr">
+        <is>
+          <t>https://exponentialroadmap.org</t>
+        </is>
+      </c>
+      <c r="L72" s="7" t="inlineStr">
+        <is>
+          <t>Initiative on exponential climate action. Named in Alexander Schmidt’s biography.</t>
+        </is>
+      </c>
+      <c r="M72" s="7" t="inlineStr">
+        <is>
+          <t>A fellowship, not his main listed job. Confirm the relationship before you email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="78" customHeight="1">
+      <c r="A73" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in a speaker bio</t>
+        </is>
+      </c>
+      <c r="B73" s="9" t="inlineStr">
+        <is>
+          <t>FrameworkESG</t>
+        </is>
+      </c>
+      <c r="C73" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G73" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H73" s="9" t="inlineStr">
+        <is>
+          <t>No current speaker. KT Michaelson was previously Managing Director.</t>
+        </is>
+      </c>
+      <c r="I73" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J73" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="K73" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="L73" s="9" t="inlineStr">
+        <is>
+          <t>ESG consultancy named in KT Michaelson’s biography.</t>
+        </is>
+      </c>
+      <c r="M73" s="9" t="inlineStr">
+        <is>
+          <t>Past employer. No website was confirmed in this pass. Her current role is at ALDI South.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="78" customHeight="1">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in a speaker bio</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>Friends of the Earth</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>No current speaker. Jonathon Porritt is a former director.</t>
+        </is>
+      </c>
+      <c r="I74" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J74" s="7" t="inlineStr">
+        <is>
+          <t>https://friendsoftheearth.org.uk</t>
+        </is>
+      </c>
+      <c r="K74" s="7" t="inlineStr">
+        <is>
+          <t>https://friendsoftheearth.org.uk</t>
+        </is>
+      </c>
+      <c r="L74" s="7" t="inlineStr">
+        <is>
+          <t>Environmental campaign group. Named in Jonathon Porritt’s biography.</t>
+        </is>
+      </c>
+      <c r="M74" s="7" t="inlineStr">
+        <is>
+          <t>Past role. His current listed affiliation is Forum for the Future.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="78" customHeight="1">
+      <c r="A75" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in a speaker bio</t>
+        </is>
+      </c>
+      <c r="B75" s="9" t="inlineStr">
+        <is>
+          <t>Global Reporting Initiative</t>
+        </is>
+      </c>
+      <c r="C75" s="9" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="E75" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G75" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H75" s="9" t="inlineStr">
+        <is>
+          <t>No current speaker. Tim Mohin is a former chief executive.</t>
+        </is>
+      </c>
+      <c r="I75" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J75" s="9" t="inlineStr">
+        <is>
+          <t>https://www.globalreporting.org</t>
+        </is>
+      </c>
+      <c r="K75" s="9" t="inlineStr">
+        <is>
+          <t>https://www.globalreporting.org</t>
+        </is>
+      </c>
+      <c r="L75" s="9" t="inlineStr">
+        <is>
+          <t>Organisation behind the GRI sustainability-reporting standards. Named in Tim Mohin’s biography.</t>
+        </is>
+      </c>
+      <c r="M75" s="9" t="inlineStr">
+        <is>
+          <t>Past role. His current role is CEO of the GHG Protocol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="78" customHeight="1">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in a speaker bio</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>Manufacture 2030</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>No current speaker. Isobel Farnsworth previously worked there on a product-carbon-footprint tool.</t>
+        </is>
+      </c>
+      <c r="I76" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J76" s="7" t="inlineStr">
+        <is>
+          <t>https://manufacture2030.com</t>
+        </is>
+      </c>
+      <c r="K76" s="7" t="inlineStr">
+        <is>
+          <t>https://manufacture2030.com</t>
+        </is>
+      </c>
+      <c r="L76" s="7" t="inlineStr">
+        <is>
+          <t>Supplier-engagement platform named in Isobel Farnsworth’s biography.</t>
+        </is>
+      </c>
+      <c r="M76" s="7" t="inlineStr">
+        <is>
+          <t>Past employer. Confirm the site is still live. Her current role is at WBCSD on PACT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="78" customHeight="1">
+      <c r="A77" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in a speaker bio</t>
+        </is>
+      </c>
+      <c r="B77" s="9" t="inlineStr">
+        <is>
+          <t>Responsible Business Alliance</t>
+        </is>
+      </c>
+      <c r="C77" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E77" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F77" s="9" t="inlineStr">
+        <is>
+          <t>Tim Mohin (founder, as stated in his speaker biography)</t>
+        </is>
+      </c>
+      <c r="G77" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H77" s="9" t="inlineStr">
+        <is>
+          <t>No current speaker from the Alliance. Tim Mohin founded it. He is now CEO of the GHG Protocol.</t>
+        </is>
+      </c>
+      <c r="I77" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J77" s="9" t="inlineStr">
+        <is>
+          <t>https://www.responsiblebusiness.org</t>
+        </is>
+      </c>
+      <c r="K77" s="9" t="inlineStr">
+        <is>
+          <t>https://www.responsiblebusiness.org</t>
+        </is>
+      </c>
+      <c r="L77" s="9" t="inlineStr">
+        <is>
+          <t>Industry coalition on responsible sourcing in global supply chains. Named in Tim Mohin’s biography.</t>
+        </is>
+      </c>
+      <c r="M77" s="9" t="inlineStr">
+        <is>
+          <t>Confirm he is still involved before you use his name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="78" customHeight="1">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in a speaker bio</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Society for the Environment</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>Not a founder-led company.</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H78" s="7" t="inlineStr">
+        <is>
+          <t>Sue Buxey is a board member and chairs its Registration Authority. Her speaking role is at ISEP.</t>
+        </is>
+      </c>
+      <c r="I78" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J78" s="7" t="inlineStr">
+        <is>
+          <t>https://socenv.org.uk</t>
+        </is>
+      </c>
+      <c r="K78" s="7" t="inlineStr">
+        <is>
+          <t>https://socenv.org.uk</t>
+        </is>
+      </c>
+      <c r="L78" s="7" t="inlineStr">
+        <is>
+          <t>Body that awards Chartered Environmentalist registration. Named in Sue Buxey’s biography.</t>
+        </is>
+      </c>
+      <c r="M78" s="7" t="inlineStr">
+        <is>
+          <t>A board role, not her main listed job.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="78" customHeight="1">
+      <c r="A79" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — named in a speaker bio</t>
+        </is>
+      </c>
+      <c r="B79" s="9" t="inlineStr">
+        <is>
+          <t>World Resources Institute</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E79" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F79" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G79" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H79" s="9" t="inlineStr">
+        <is>
+          <t>No current speaker. Laura Draucker previously worked on the GHG Protocol team there.</t>
+        </is>
+      </c>
+      <c r="I79" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J79" s="9" t="inlineStr">
+        <is>
+          <t>https://www.wri.org</t>
+        </is>
+      </c>
+      <c r="K79" s="9" t="inlineStr">
+        <is>
+          <t>https://www.wri.org</t>
+        </is>
+      </c>
+      <c r="L79" s="9" t="inlineStr">
+        <is>
+          <t>Environmental research organisation. The GHG Protocol was developed with WRI. Named in Laura Draucker’s biography.</t>
+        </is>
+      </c>
+      <c r="M79" s="9" t="inlineStr">
+        <is>
+          <t>Past employer. Her current role is at the Center for Green Market Activation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="78" customHeight="1">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — participant list</t>
+        </is>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>ARPenviro</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>Bratislava</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>Slovakia</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>English and Slovak</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H80" s="7" t="inlineStr">
+        <is>
+          <t>From the participant list. Find the person who attended before you email.</t>
+        </is>
+      </c>
+      <c r="I80" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J80" s="7" t="inlineStr">
+        <is>
+          <t>https://arpenviro.com/en/</t>
+        </is>
+      </c>
+      <c r="K80" s="7" t="inlineStr">
+        <is>
+          <t>https://arpenviro.com/en/</t>
+        </is>
+      </c>
+      <c r="L80" s="7" t="inlineStr">
+        <is>
+          <t>Slovak environmental consultancy focused on air protection, greenhouse-gas verification, carbon footprints, and LCA.</t>
+        </is>
+      </c>
+      <c r="M80" s="7" t="inlineStr">
+        <is>
+          <t>You identified this name on the CAA participant list. The English site is arpenviro.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="78" customHeight="1">
+      <c r="A81" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — participant list</t>
+        </is>
+      </c>
+      <c r="B81" s="9" t="inlineStr">
+        <is>
+          <t>Catalyst Commercial</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F81" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G81" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H81" s="9" t="inlineStr">
+        <is>
+          <t>From the participant list. Find the person who attended before you email.</t>
+        </is>
+      </c>
+      <c r="I81" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J81" s="9" t="inlineStr">
+        <is>
+          <t>https://www.catalyst-commercial.co.uk</t>
+        </is>
+      </c>
+      <c r="K81" s="9" t="inlineStr">
+        <is>
+          <t>https://www.catalyst-commercial.co.uk/carbon-reporting/</t>
+        </is>
+      </c>
+      <c r="L81" s="9" t="inlineStr">
+        <is>
+          <t>UK energy and carbon consultancy. Carbon reporting runs through its EaaSi Carbon platform.</t>
+        </is>
+      </c>
+      <c r="M81" s="9" t="inlineStr">
+        <is>
+          <t>You identified this name on the CAA participant list. The legal name on its carbon-reduction plan is Catalyst Commercial Services Limited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="78" customHeight="1">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — participant list</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>Ekos Plus</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>Bratislava</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>Slovakia</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>Slovak</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H82" s="7" t="inlineStr">
+        <is>
+          <t>From the participant list. Find the person who attended before you email.</t>
+        </is>
+      </c>
+      <c r="I82" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J82" s="7" t="inlineStr">
+        <is>
+          <t>https://www.ekosplus.sk</t>
+        </is>
+      </c>
+      <c r="K82" s="7" t="inlineStr">
+        <is>
+          <t>https://www.ekosplus.sk</t>
+        </is>
+      </c>
+      <c r="L82" s="7" t="inlineStr">
+        <is>
+          <t>Slovak environmental consultancy, including greenhouse-gas emissions verification and environmental permitting. Not the New Zealand firm Ekos.</t>
+        </is>
+      </c>
+      <c r="M82" s="7" t="inlineStr">
+        <is>
+          <t>You identified this name on the CAA participant list. The public site is in Slovak. It also runs a CARBON DAY conference in Bratislava.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="78" customHeight="1">
+      <c r="A83" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — participant list</t>
+        </is>
+      </c>
+      <c r="B83" s="9" t="inlineStr">
+        <is>
+          <t>Environmental Strategies Limited</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>Selby</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E83" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F83" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G83" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H83" s="9" t="inlineStr">
+        <is>
+          <t>Helen Sprakes is Managing Director on the company site. Confirm she is the right contact. The participant-list attendee was not named.</t>
+        </is>
+      </c>
+      <c r="I83" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J83" s="9" t="inlineStr">
+        <is>
+          <t>https://esltd.co.uk</t>
+        </is>
+      </c>
+      <c r="K83" s="9" t="inlineStr">
+        <is>
+          <t>https://esltd.co.uk/our-clients/verification/</t>
+        </is>
+      </c>
+      <c r="L83" s="9" t="inlineStr">
+        <is>
+          <t>UK energy and environmental consultancy. It verifies greenhouse-gas inventories and supports carbon reporting.</t>
+        </is>
+      </c>
+      <c r="M83" s="9" t="inlineStr">
+        <is>
+          <t>You identified this name on the CAA participant list. This is the Selby firm at esltd.co.uk, not Environmental Strategies International in Los Angeles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="78" customHeight="1">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — participant list</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>FuturePlus</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F84" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G84" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H84" s="7" t="inlineStr">
+        <is>
+          <t>From the participant list. Find the person who attended before you email.</t>
+        </is>
+      </c>
+      <c r="I84" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J84" s="7" t="inlineStr">
+        <is>
+          <t>https://future-plus.co.uk</t>
+        </is>
+      </c>
+      <c r="K84" s="7" t="inlineStr">
+        <is>
+          <t>https://future-plus.co.uk</t>
+        </is>
+      </c>
+      <c r="L84" s="7" t="inlineStr">
+        <is>
+          <t>Sustainability and ESG platform for assessing, planning, and reporting.</t>
+        </is>
+      </c>
+      <c r="M84" s="7" t="inlineStr">
+        <is>
+          <t>You identified this name on the CAA participant list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="78" customHeight="1">
+      <c r="A85" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — participant list</t>
+        </is>
+      </c>
+      <c r="B85" s="9" t="inlineStr">
+        <is>
+          <t>ICON Carbon</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="inlineStr">
+        <is>
+          <t>Manchester</t>
+        </is>
+      </c>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E85" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F85" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G85" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H85" s="9" t="inlineStr">
+        <is>
+          <t>Tony Summers is Director on a public profile. Confirm he attended, and that this is the ICON on the participant list.</t>
+        </is>
+      </c>
+      <c r="I85" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J85" s="9" t="inlineStr">
+        <is>
+          <t>https://iconcarbon.co.uk</t>
+        </is>
+      </c>
+      <c r="K85" s="9" t="inlineStr">
+        <is>
+          <t>https://iconcarbon.co.uk</t>
+        </is>
+      </c>
+      <c r="L85" s="9" t="inlineStr">
+        <is>
+          <t>UK consultancy for carbon reporting and compliance, including UK ETS, SECR, and ISO 50001.</t>
+        </is>
+      </c>
+      <c r="M85" s="9" t="inlineStr">
+        <is>
+          <t>The participant list said ICON. This row is ICON Carbon Ltd. Confirm it is the same organisation before you email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="78" customHeight="1">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — participant list</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Impatience Earth</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F86" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G86" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H86" s="7" t="inlineStr">
+        <is>
+          <t>From the participant list. Find the person who attended before you email.</t>
+        </is>
+      </c>
+      <c r="I86" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J86" s="7" t="inlineStr">
+        <is>
+          <t>https://impatience.earth</t>
+        </is>
+      </c>
+      <c r="K86" s="7" t="inlineStr">
+        <is>
+          <t>https://impatience.earth</t>
+        </is>
+      </c>
+      <c r="L86" s="7" t="inlineStr">
+        <is>
+          <t>Nonprofit climate consultancy for funders, businesses, and agriculture-linked supply chains.</t>
+        </is>
+      </c>
+      <c r="M86" s="7" t="inlineStr">
+        <is>
+          <t>You identified this name on the CAA participant list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="78" customHeight="1">
+      <c r="A87" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — participant list</t>
+        </is>
+      </c>
+      <c r="B87" s="9" t="inlineStr">
+        <is>
+          <t>MyCarbon</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D87" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E87" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F87" s="9" t="inlineStr">
+        <is>
+          <t>Toby and Mike are named as co-founders on the about page. Surnames were not copied here. Confirm them on the site.</t>
+        </is>
+      </c>
+      <c r="G87" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H87" s="9" t="inlineStr">
+        <is>
+          <t>From the participant list. Find the person who attended before you email.</t>
+        </is>
+      </c>
+      <c r="I87" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J87" s="9" t="inlineStr">
+        <is>
+          <t>https://www.mycarbon.co.uk</t>
+        </is>
+      </c>
+      <c r="K87" s="9" t="inlineStr">
+        <is>
+          <t>https://www.mycarbon.co.uk/about-us/</t>
+        </is>
+      </c>
+      <c r="L87" s="9" t="inlineStr">
+        <is>
+          <t>UK carbon-management consultancy for footprints, reduction plans, and offsetting. The legal name on the site is Carbon Green Limited.</t>
+        </is>
+      </c>
+      <c r="M87" s="9" t="inlineStr">
+        <is>
+          <t>You identified this name on the CAA participant list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="78" customHeight="1">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — participant list</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>Positive Planet</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F88" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G88" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H88" s="7" t="inlineStr">
+        <is>
+          <t>From the participant list. Find the person who attended before you email.</t>
+        </is>
+      </c>
+      <c r="I88" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J88" s="7" t="inlineStr">
+        <is>
+          <t>https://positiveplanet.uk</t>
+        </is>
+      </c>
+      <c r="K88" s="7" t="inlineStr">
+        <is>
+          <t>https://positiveplanet.uk/esg/</t>
+        </is>
+      </c>
+      <c r="L88" s="7" t="inlineStr">
+        <is>
+          <t>UK sustainability advisory firm for carbon measurement, reduction, training, and ESG reporting.</t>
+        </is>
+      </c>
+      <c r="M88" s="7" t="inlineStr">
+        <is>
+          <t>You identified this name on the CAA participant list. A Manchester phone number is on the site. Confirm the office.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="78" customHeight="1">
+      <c r="A89" s="9" t="inlineStr">
+        <is>
+          <t>CAA 2026 — participant list</t>
+        </is>
+      </c>
+      <c r="B89" s="9" t="inlineStr">
+        <is>
+          <t>Sagana</t>
+        </is>
+      </c>
+      <c r="C89" s="9" t="inlineStr">
+        <is>
+          <t>Zurich</t>
+        </is>
+      </c>
+      <c r="D89" s="9" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E89" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F89" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G89" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H89" s="9" t="inlineStr">
+        <is>
+          <t>From the participant list. Find the person who attended before you email.</t>
+        </is>
+      </c>
+      <c r="I89" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J89" s="9" t="inlineStr">
+        <is>
+          <t>https://sagana.com</t>
+        </is>
+      </c>
+      <c r="K89" s="9" t="inlineStr">
+        <is>
+          <t>https://sagana.com</t>
+        </is>
+      </c>
+      <c r="L89" s="9" t="inlineStr">
+        <is>
+          <t>Impact and climate-strategy firm. It works with companies and foundations on decarbonisation and climate-related investment.</t>
+        </is>
+      </c>
+      <c r="M89" s="9" t="inlineStr">
+        <is>
+          <t>You identified this name on the CAA participant list. Zurich is the location shown on the site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="78" customHeight="1">
+      <c r="A90" s="7" t="inlineStr">
+        <is>
+          <t>CAA 2026 — participant list</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>SmartCarbon</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F90" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G90" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H90" s="7" t="inlineStr">
+        <is>
+          <t>From the participant list. Find the person who attended before you email.</t>
+        </is>
+      </c>
+      <c r="I90" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J90" s="7" t="inlineStr">
+        <is>
+          <t>https://www.smartcarboncalculator.com</t>
+        </is>
+      </c>
+      <c r="K90" s="7" t="inlineStr">
+        <is>
+          <t>https://www.smartcarboncalculator.com/carbon-emissions-consulting/</t>
+        </is>
+      </c>
+      <c r="L90" s="7" t="inlineStr">
+        <is>
+          <t>UK carbon-accounting platform plus consultancy for measurement, reporting, and supply-chain emissions.</t>
+        </is>
+      </c>
+      <c r="M90" s="7" t="inlineStr">
+        <is>
+          <t>You identified this name on the CAA participant list. Use smartcarboncalculator.com. smartcarbon.co.uk was for sale when checked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="78" customHeight="1">
+      <c r="A91" s="9" t="inlineStr">
+        <is>
+          <t>Added by you</t>
+        </is>
+      </c>
+      <c r="B91" s="9" t="inlineStr">
+        <is>
+          <t>Gold Standard</t>
+        </is>
+      </c>
+      <c r="C91" s="9" t="inlineStr">
+        <is>
+          <t>Geneva</t>
+        </is>
+      </c>
+      <c r="D91" s="9" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E91" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F91" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G91" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H91" s="9" t="inlineStr">
+        <is>
+          <t>Not taken from the speaker list. Find the current content or methodology contact.</t>
+        </is>
+      </c>
+      <c r="I91" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J91" s="9" t="inlineStr">
+        <is>
+          <t>https://www.goldstandard.org</t>
+        </is>
+      </c>
+      <c r="K91" s="9" t="inlineStr">
+        <is>
+          <t>https://www.goldstandard.org</t>
+        </is>
+      </c>
+      <c r="L91" s="9" t="inlineStr">
+        <is>
+          <t>Standard-setting and certification body for carbon credits that also measures wider sustainable-development impact.</t>
+        </is>
+      </c>
+      <c r="M91" s="9" t="inlineStr">
+        <is>
+          <t>You asked for this row. The Center for Green Market Activation describes the AIM Platform as a partnership with Gold Standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="78" customHeight="1">
+      <c r="A92" s="7" t="inlineStr">
+        <is>
+          <t>Added by you</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>KBR</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G92" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H92" s="7" t="inlineStr">
+        <is>
+          <t>Not taken from the speaker list. Find the sustainability or marketing contact.</t>
+        </is>
+      </c>
+      <c r="I92" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J92" s="7" t="inlineStr">
+        <is>
+          <t>https://www.kbr.com</t>
+        </is>
+      </c>
+      <c r="K92" s="7" t="inlineStr">
+        <is>
+          <t>https://www.kbr.com</t>
+        </is>
+      </c>
+      <c r="L92" s="7" t="inlineStr">
+        <is>
+          <t>US engineering, technology, and government-services company working in energy transition, defence, and space.</t>
+        </is>
+      </c>
+      <c r="M92" s="7" t="inlineStr">
+        <is>
+          <t>You asked for this row. A company of this size will have its own communications team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="78" customHeight="1">
+      <c r="A93" s="9" t="inlineStr">
+        <is>
+          <t>Added by you</t>
+        </is>
+      </c>
+      <c r="B93" s="9" t="inlineStr">
+        <is>
+          <t>Planet Mark</t>
+        </is>
+      </c>
+      <c r="C93" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D93" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E93" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F93" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G93" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H93" s="9" t="inlineStr">
+        <is>
+          <t>Matt Letley, now founder of UK Carbon Verification, was previously Commercial Director. Find the current Planet Mark contact.</t>
+        </is>
+      </c>
+      <c r="I93" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J93" s="9" t="inlineStr">
+        <is>
+          <t>https://www.planetmark.com</t>
+        </is>
+      </c>
+      <c r="K93" s="9" t="inlineStr">
+        <is>
+          <t>https://www.planetmark.com</t>
+        </is>
+      </c>
+      <c r="L93" s="9" t="inlineStr">
+        <is>
+          <t>UK sustainability certification body and consultancy that helps organisations measure and cut their carbon footprint.</t>
+        </is>
+      </c>
+      <c r="M93" s="9" t="inlineStr">
+        <is>
+          <t>You asked for this row. It is also named in Matt Letley’s CAA speaker biography as a past employer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="78" customHeight="1">
+      <c r="A94" s="7" t="inlineStr">
+        <is>
+          <t>Added by you</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>Seaway7</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G94" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H94" s="7" t="inlineStr">
+        <is>
+          <t>Not taken from the speaker list. Find the sustainability contact. It is the offshore-wind business of Subsea7.</t>
+        </is>
+      </c>
+      <c r="I94" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J94" s="7" t="inlineStr">
+        <is>
+          <t>https://www.seaway7.com</t>
+        </is>
+      </c>
+      <c r="K94" s="7" t="inlineStr">
+        <is>
+          <t>https://www.seaway7.com</t>
+        </is>
+      </c>
+      <c r="L94" s="7" t="inlineStr">
+        <is>
+          <t>Offshore wind installation and foundation business of Subsea7.</t>
+        </is>
+      </c>
+      <c r="M94" s="7" t="inlineStr">
+        <is>
+          <t>You asked for this row. Check whether a Subsea7–Saipem merger changes the name before you write.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="78" customHeight="1">
+      <c r="A95" s="9" t="inlineStr">
+        <is>
+          <t>Added by you</t>
+        </is>
+      </c>
+      <c r="B95" s="9" t="inlineStr">
+        <is>
+          <t>Subsea7</t>
+        </is>
+      </c>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="D95" s="9" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="E95" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F95" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G95" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H95" s="9" t="inlineStr">
+        <is>
+          <t>Not taken from the speaker list. Find the sustainability contact.</t>
+        </is>
+      </c>
+      <c r="I95" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J95" s="9" t="inlineStr">
+        <is>
+          <t>https://www.subsea7.com</t>
+        </is>
+      </c>
+      <c r="K95" s="9" t="inlineStr">
+        <is>
+          <t>https://www.subsea7.com</t>
+        </is>
+      </c>
+      <c r="L95" s="9" t="inlineStr">
+        <is>
+          <t>Offshore engineering and construction contractor for oil and gas and for renewables.</t>
+        </is>
+      </c>
+      <c r="M95" s="9" t="inlineStr">
+        <is>
+          <t>You asked for this row. The announced merger with Saipem had not completed as of early October 2026. The European Commission’s Phase II review was still open after the clock stopped on 25 August 2026, and Australia was also in Phase II. Saipem’s CEO said on 29 September 2026 that 10 of 16 authorities had cleared it. Treat Subsea7 as a separate company until the merger closes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="78" customHeight="1">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
+          <t>Added by you</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>TP ICAP</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F96" s="7" t="inlineStr">
+        <is>
+          <t>Not confirmed in the sources checked for this list</t>
+        </is>
+      </c>
+      <c r="G96" s="7" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H96" s="7" t="inlineStr">
+        <is>
+          <t>Not taken from the speaker list. Find the sustainability or marketing contact.</t>
+        </is>
+      </c>
+      <c r="I96" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J96" s="7" t="inlineStr">
+        <is>
+          <t>https://www.tpicap.com</t>
+        </is>
+      </c>
+      <c r="K96" s="7" t="inlineStr">
+        <is>
+          <t>https://www.tpicap.com</t>
+        </is>
+      </c>
+      <c r="L96" s="7" t="inlineStr">
+        <is>
+          <t>Interdealer broker and market-data group, which also operates in energy and environmental markets.</t>
+        </is>
+      </c>
+      <c r="M96" s="7" t="inlineStr">
+        <is>
+          <t>You asked for this row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="78" customHeight="1">
+      <c r="A97" s="9" t="inlineStr">
+        <is>
+          <t>Added by you</t>
+        </is>
+      </c>
+      <c r="B97" s="9" t="inlineStr">
+        <is>
+          <t>Willmott Dixon</t>
+        </is>
+      </c>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>Confirm on the site</t>
+        </is>
+      </c>
+      <c r="D97" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E97" s="9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F97" s="9" t="inlineStr">
+        <is>
+          <t>Not a founder-led company in the sources checked. It is privately owned.</t>
+        </is>
+      </c>
+      <c r="G97" s="9" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="H97" s="9" t="inlineStr">
+        <is>
+          <t>Not taken from the speaker list. Find the sustainability contact.</t>
+        </is>
+      </c>
+      <c r="I97" s="13" t="inlineStr">
+        <is>
+          <t>Not scored</t>
+        </is>
+      </c>
+      <c r="J97" s="9" t="inlineStr">
+        <is>
+          <t>https://www.willmottdixon.co.uk</t>
+        </is>
+      </c>
+      <c r="K97" s="9" t="inlineStr">
+        <is>
+          <t>https://www.willmottdixon.co.uk</t>
+        </is>
+      </c>
+      <c r="L97" s="9" t="inlineStr">
+        <is>
+          <t>Privately owned UK construction and property-services contractor with a sustainability and social-value agenda.</t>
+        </is>
+      </c>
+      <c r="M97" s="9" t="inlineStr">
+        <is>
+          <t>You asked for this row.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M30"/>
+  <autoFilter ref="A1:M97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>